<commit_message>
Subscriptions system, PDF records export, Understat xG features + xG-Poisson model, live preview dashboard
</commit_message>
<xml_diff>
--- a/records/exports/records.xlsx
+++ b/records/exports/records.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="Users" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Rewards" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Invoices" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Predictions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Results" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Model Performance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Subscriptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Invoices" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Predictions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Model Performance" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Predictions'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Predictions'!$A$1:$J$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -567,6 +568,68 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002ECC71"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Subscription ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Started</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unlocked By Points</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Benefits</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001B2A4A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -626,7 +689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001B2A4A"/>
@@ -755,7 +818,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001B2A4A"/>
@@ -835,7 +898,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002ECC71"/>

</xml_diff>

<commit_message>
Vendicator rename, glass/neon UI, 6-league sweep + UCL/UEL, draw head, injuries adapter, temporal prototype, WP plugin deployed to staging
</commit_message>
<xml_diff>
--- a/records/exports/records.xlsx
+++ b/records/exports/records.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Model Performance" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Users'!$A$1:$J$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Predictions'!$A$1:$J$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,12 +443,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -509,8 +510,68 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>claudio</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>bluetuxedo808@proton.me</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eljay00p@gmail.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>eljay00p@gmail.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -560,7 +621,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -622,7 +683,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -684,7 +745,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -812,7 +873,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
   <autoFilter ref="A1:J2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -893,7 +954,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -943,7 +1004,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A095"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Player markets with last-5 dot tallies and value-based points, discipline markets, canonical team registry, league tables + player profiles, per-competition market config, dashboard filtering/paging and hover layering fixes
</commit_message>
<xml_diff>
--- a/records/exports/records.xlsx
+++ b/records/exports/records.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Users'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Predictions'!$A$1:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Predictions'!$A$1:$J$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -757,12 +757,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -1236,9 +1236,4481 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T12:24:54.185463+00:00</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sheffield Weds vs Bradford</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>20/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 49.0, "draw": 23.8, "away": 27.1}</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 49.0, "draw": 23.8, "away": 27.1}</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-21T12:26:04.678647+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ath Madrid vs Malaga</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>19/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>{"home": 75.9, "draw": 13.1, "away": 11.0}</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>{"home": 75.9, "draw": 13.1, "away": 11.0}</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T12:26:04.722036+00:00</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Vallecano vs Alaves</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>20/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 47.8, "draw": 33.5, "away": 18.7}</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 47.8, "draw": 33.5, "away": 18.7}</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:15.212773+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Hull City vs Manchester United</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>22/08/2026 12:30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>{"home": 17.0, "draw": 15.2, "away": 67.8}</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>{"home": 17.0, "draw": 15.2, "away": 67.8}</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:22.886878+00:00</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Everton vs Crystal Palace</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 44.4, "draw": 24.4, "away": 31.1}</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 44.4, "draw": 24.4, "away": 31.1}</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:26.007357+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ipswich Town vs Sunderland</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>{"home": 39.3, "draw": 19.4, "away": 41.2}</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>{"home": 39.3, "draw": 19.4, "away": 41.2}</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:29.497630+00:00</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Nottingham Forest vs Leeds United</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 44.4, "draw": 24.4, "away": 31.1}</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 44.4, "draw": 24.4, "away": 31.1}</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:37.294672+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Brentford vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>22/08/2026 17:30</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>{"home": 43.5, "draw": 26.0, "away": 30.5}</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>{"home": 43.5, "draw": 26.0, "away": 30.5}</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:44.208457+00:00</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 14:00</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 44.7, "draw": 23.9, "away": 31.3}</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 44.7, "draw": 23.9, "away": 31.3}</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:51.485400+00:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Manchester City vs Bournemouth</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>23/08/2026 14:00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>{"home": 59.2, "draw": 20.2, "away": 20.6}</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>{"home": 59.2, "draw": 20.2, "away": 20.6}</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:17:58.937424+00:00</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle United vs Liverpool</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 16:30</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 31.6, "draw": 21.9, "away": 46.5}</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 31.6, "draw": 21.9, "away": 46.5}</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:18:06.736556+00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>E0</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Fulham vs Chelsea</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>24/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>{"home": 31.6, "draw": 21.9, "away": 46.5}</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>{"home": 31.6, "draw": 21.9, "away": 46.5}</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:00.805387+00:00</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Birmingham City vs Bristol City</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 12:30</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 56.8, "draw": 25.8, "away": 17.4}</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 56.8, "draw": 25.8, "away": 17.4}</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:00.849205+00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Millwall vs Norwich City</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>22/08/2026 12:30</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>{"home": 40.4, "draw": 30.3, "away": 29.3}</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>{"home": 40.4, "draw": 30.3, "away": 29.3}</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:00.896206+00:00</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Blackburn Rovers vs Middlesbrough</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 23.6, "draw": 39.2, "away": 37.3}</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 23.6, "draw": 39.2, "away": 37.3}</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:00.942801+00:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Derby County vs Cardiff City</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>{"home": 43.7, "draw": 26.4, "away": 29.9}</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>{"home": 43.7, "draw": 26.4, "away": 29.9}</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:00.986949+00:00</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Preston North End vs Wolverhampton Wanderers</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 19.1, "draw": 41.5, "away": 39.4}</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 19.1, "draw": 41.5, "away": 39.4}</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:01.034312+00:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Queens Park Rangers vs Bolton</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>{"home": 50.2, "draw": 23.4, "away": 26.4}</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>{"home": 50.2, "draw": 23.4, "away": 26.4}</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:01.078043+00:00</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Southampton vs Stoke City</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 61.8, "draw": 20.5, "away": 17.8}</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 61.8, "draw": 20.5, "away": 17.8}</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:01.123974+00:00</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Swansea City vs Sheffield United</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>{"home": 35.3, "draw": 30.7, "away": 34.0}</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>{"home": 35.3, "draw": 30.7, "away": 34.0}</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:01.169836+00:00</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Wrexham vs Watford</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.0, "draw": 25.3, "away": 28.7}</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.0, "draw": 25.3, "away": 28.7}</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:20:01.216011+00:00</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion vs Burnley</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>23/08/2026 12:00</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>{"home": 35.0, "draw": 39.1, "away": 25.8}</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>{"home": 35.0, "draw": 39.1, "away": 25.8}</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.281486+00:00</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Doncaster vs Barnsley</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 12:30</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.5, "draw": 22.6, "away": 30.9}</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.5, "draw": 22.6, "away": 30.9}</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.328655+00:00</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>AFC Wimbledon vs Reading</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>{"home": 34.8, "draw": 26.7, "away": 38.5}</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>{"home": 34.8, "draw": 26.7, "away": 38.5}</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.379087+00:00</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Milton Keynes Dons vs Huddersfield</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.3, "draw": 23.0, "away": 35.7}</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.3, "draw": 23.0, "away": 35.7}</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.426608+00:00</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Peterboro vs Mansfield</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>{"home": 33.6, "draw": 30.2, "away": 36.2}</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>{"home": 33.6, "draw": 30.2, "away": 36.2}</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.472722+00:00</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Stevenage vs Oxford United</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 43.7, "draw": 23.8, "away": 32.5}</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 43.7, "draw": 23.8, "away": 32.5}</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.524397+00:00</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Stockport vs Blackpool</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>{"home": 54.1, "draw": 25.7, "away": 20.2}</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>{"home": 54.1, "draw": 25.7, "away": 20.2}</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.574403+00:00</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Wigan vs Leyton Orient</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.5, "draw": 22.6, "away": 30.9}</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.5, "draw": 22.6, "away": 30.9}</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:21:55.619904+00:00</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Wycombe vs Plymouth</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>{"home": 40.3, "draw": 29.1, "away": 30.7}</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>{"home": 40.3, "draw": 29.1, "away": 30.7}</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:44.919005+00:00</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Bristol Rvs vs Newport County</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 12:30</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.7, "draw": 29.7, "away": 23.6}</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.7, "draw": 29.7, "away": 23.6}</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:44.962584+00:00</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Salford vs Chesterfield</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>22/08/2026 12:30</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>{"home": 34.8, "draw": 31.4, "away": 33.9}</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>{"home": 34.8, "draw": 31.4, "away": 33.9}</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.006952+00:00</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Walsall vs Grimsby</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 12:30</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 26.6, "draw": 30.6, "away": 42.8}</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 26.6, "draw": 30.6, "away": 42.8}</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.052265+00:00</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Colchester vs Oldham</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>{"home": 33.5, "draw": 30.2, "away": 36.2}</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>{"home": 33.5, "draw": 30.2, "away": 36.2}</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.095947+00:00</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Crewe vs Northampton</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 34.8, "draw": 31.4, "away": 33.9}</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 34.8, "draw": 31.4, "away": 33.9}</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.141068+00:00</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Exeter vs Accrington</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>{"home": 43.3, "draw": 31.1, "away": 25.6}</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>{"home": 43.3, "draw": 31.1, "away": 25.6}</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.185504+00:00</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Fleetwood Town vs Gillingham</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 39.1, "draw": 29.7, "away": 31.2}</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 39.1, "draw": 29.7, "away": 31.2}</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.228872+00:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Port Vale vs Tranmere</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>{"home": 53.1, "draw": 30.2, "away": 16.7}</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>{"home": 53.1, "draw": 30.2, "away": 16.7}</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.273271+00:00</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Rochdale vs Crawley Town</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 39.1, "draw": 29.7, "away": 31.2}</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 39.1, "draw": 29.7, "away": 31.2}</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.317663+00:00</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Shrewsbury vs Barnet</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>{"home": 24.8, "draw": 33.7, "away": 41.5}</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>{"home": 24.8, "draw": 33.7, "away": 41.5}</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:23:45.361836+00:00</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Swindon vs Cheltenham</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 15:00</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 39.6, "draw": 29.5, "away": 31.0}</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 39.6, "draw": 29.5, "away": 31.0}</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:24:58.901520+00:00</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Marseille vs Strasbourg</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>21/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>{"home": 46.9, "draw": 25.1, "away": 28.0}</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>{"home": 46.9, "draw": 25.1, "away": 28.0}</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:25:06.893443+00:00</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Lens vs Auxerre</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 16:15</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 61.2, "draw": 18.5, "away": 20.3}</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 61.2, "draw": 18.5, "away": 20.3}</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:25:10.880024+00:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Nice vs Lorient</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>22/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>{"home": 42.8, "draw": 31.0, "away": 26.2}</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>{"home": 42.8, "draw": 31.0, "away": 26.2}</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:25:18.786490+00:00</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Toulouse vs Lyon</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 28.6, "draw": 25.6, "away": 45.9}</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 28.6, "draw": 25.6, "away": 45.9}</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:25:18.831805+00:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Troyes vs Paris FC</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>22/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>{"home": 24.4, "draw": 31.5, "away": 44.1}</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>{"home": 24.4, "draw": 31.5, "away": 44.1}</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:25:26.051337+00:00</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Angers vs Lille</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 14:00</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 18.7, "draw": 31.7, "away": 49.6}</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 18.7, "draw": 31.7, "away": 49.6}</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:25:33.607070+00:00</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Le Havre vs Monaco</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>23/08/2026 16:15</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>{"home": 20.4, "draw": 25.5, "away": 54.1}</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>{"home": 20.4, "draw": 25.5, "away": 54.1}</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:25:37.292563+00:00</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain vs Rennes</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 62.5, "draw": 16.8, "away": 20.7}</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 62.5, "draw": 16.8, "away": 20.7}</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:26:58.671539+00:00</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Inter Milan vs Monza</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>22/08/2026 17:30</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>{"home": 92.7, "draw": 0.0, "away": 7.3}</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>{"home": 92.7, "draw": 0.0, "away": 7.3}</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:06.782498+00:00</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Udinese vs Como</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 17:30</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 21.3, "draw": 29.8, "away": 48.8}</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 21.3, "draw": 29.8, "away": 48.8}</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:16.117688+00:00</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Genoa vs Napoli</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>22/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>{"home": 22.6, "draw": 25.8, "away": 51.7}</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>{"home": 22.6, "draw": 25.8, "away": 51.7}</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:20.207351+00:00</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Parma vs Cagliari</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.5, "draw": 33.0, "away": 25.6}</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.5, "draw": 33.0, "away": 25.6}</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:24.051998+00:00</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Frosinone vs Juventus</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>23/08/2026 17:30</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>{"home": 6.1, "draw": 29.9, "away": 64.0}</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>{"home": 6.1, "draw": 29.9, "away": 64.0}</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:30.899937+00:00</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Venezia vs Lecce</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 17:30</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.9, "draw": 32.2, "away": 25.9}</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.9, "draw": 32.2, "away": 25.9}</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:35.360957+00:00</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Atalanta vs Sassuolo</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>23/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>{"home": 72.9, "draw": 16.5, "away": 10.5}</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>{"home": 72.9, "draw": 16.5, "away": 10.5}</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:43.993610+00:00</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Torino vs AC Milan</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 21.3, "draw": 29.8, "away": 48.8}</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 21.3, "draw": 29.8, "away": 48.8}</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:27:52.100571+00:00</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Bologna vs Lazio</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>24/08/2026 17:30</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>{"home": 43.6, "draw": 31.2, "away": 25.1}</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>{"home": 43.6, "draw": 31.2, "away": 25.1}</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:28:00.902086+00:00</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>AS Roma vs Fiorentina</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 19:45</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 67.3, "draw": 23.0, "away": 9.7}</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 67.3, "draw": 23.0, "away": 9.7}</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:16.843913+00:00</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catanzaro</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>21/08/2026 19:30</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>{"home": 31.0, "draw": 35.1, "away": 33.9}</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>{"home": 31.0, "draw": 35.1, "away": 33.9}</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:16.886412+00:00</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Carrarese vs Mantova</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 35.9, "draw": 24.8, "away": 39.3}</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 35.9, "draw": 24.8, "away": 39.3}</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:16.930074+00:00</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Sudtirol vs Virtus Entella</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>22/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>{"home": 39.8, "draw": 23.7, "away": 36.5}</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>{"home": 39.8, "draw": 23.7, "away": 36.5}</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:16.976129+00:00</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Benevento vs Modena</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 37.7, "draw": 24.1, "away": 38.2}</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 37.7, "draw": 24.1, "away": 38.2}</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:17.020243+00:00</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Empoli vs Cremonese</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>22/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>{"home": 34.2, "draw": 23.6, "away": 42.3}</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>{"home": 34.2, "draw": 23.6, "away": 42.3}</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:17.065050+00:00</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Pisa vs Padova</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 59.4, "draw": 15.0, "away": 25.7}</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 59.4, "draw": 15.0, "away": 25.7}</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:17.110043+00:00</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Verona vs Ascoli</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>23/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>{"home": 62.6, "draw": 15.8, "away": 21.6}</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>{"home": 62.6, "draw": 15.8, "away": 21.6}</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:17.153038+00:00</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Cesena vs Sampdoria</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 35.9, "draw": 24.8, "away": 39.3}</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 35.9, "draw": 24.8, "away": 39.3}</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:29:17.197452+00:00</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Palermo vs Juve Stabia</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>23/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>{"home": 62.6, "draw": 15.8, "away": 21.6}</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>{"home": 62.6, "draw": 15.8, "away": 21.6}</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:30:40.121750+00:00</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Real Betis vs Real Sociedad</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>21/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 52.2, "draw": 27.3, "away": 20.5}</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 52.2, "draw": 27.3, "away": 20.5}</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:30:48.853635+00:00</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Athletic Bilbao vs Sevilla</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>22/08/2026 16:00</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>{"home": 55.9, "draw": 25.2, "away": 18.9}</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>{"home": 55.9, "draw": 25.2, "away": 18.9}</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:30:56.705553+00:00</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Valencia vs Celta Vigo</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 18:30</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.9, "draw": 34.0, "away": 19.0}</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 46.9, "draw": 34.0, "away": 19.0}</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:31:05.247080+00:00</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Espanyol vs Real Madrid</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>22/08/2026 20:30</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>{"home": 13.6, "draw": 39.0, "away": 47.3}</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>{"home": 13.6, "draw": 39.0, "away": 47.3}</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:31:14.418743+00:00</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Atletico Madrid vs Villarreal</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 16:00</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 52.1, "draw": 27.4, "away": 20.4}</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 52.1, "draw": 27.4, "away": 20.4}</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:31:19.288687+00:00</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Elche vs Barcelona</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>23/08/2026 20:30</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>{"home": 14.7, "draw": 30.7, "away": 54.7}</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>{"home": 14.7, "draw": 30.7, "away": 54.7}</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:31:23.356127+00:00</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Osasuna vs Levante</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 18:30</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 47.8, "draw": 33.5, "away": 18.7}</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 47.8, "draw": 33.5, "away": 18.7}</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:31:23.408299+00:00</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Malaga vs La Coruna</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>24/08/2026 20:30</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>{"home": 41.9, "draw": 31.4, "away": 26.7}</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>{"home": 41.9, "draw": 31.4, "away": 26.7}</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:03.791929+00:00</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Cordoba vs Girona</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>21/08/2026 20:00</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 21.6, "draw": 42.7, "away": 35.7}</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 21.6, "draw": 42.7, "away": 35.7}</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:03.837262+00:00</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Oviedo vs Leganes</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>22/08/2026 16:00</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>{"home": 57.4, "draw": 25.6, "away": 17.0}</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>{"home": 57.4, "draw": 25.6, "away": 17.0}</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:03.881593+00:00</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Albacete vs Sociedad B</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 57.4, "draw": 25.6, "away": 17.0}</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 57.4, "draw": 25.6, "away": 17.0}</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:03.928385+00:00</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Ceuta vs Las Palmas</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>22/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>{"home": 17.9, "draw": 35.4, "away": 46.7}</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>{"home": 17.9, "draw": 35.4, "away": 46.7}</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:03.972230+00:00</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Eldense vs Cadiz</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026 20:30</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.5, "draw": 36.1, "away": 22.4}</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 41.5, "draw": 36.1, "away": 22.4}</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:04.017593+00:00</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Eibar vs Valladolid</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>23/08/2026 16:00</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>{"home": 52.5, "draw": 26.4, "away": 21.1}</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>{"home": 52.5, "draw": 26.4, "away": 21.1}</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:04.064828+00:00</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Castellon vs Sabadell</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 66.3, "draw": 19.9, "away": 13.8}</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 66.3, "draw": 19.9, "away": 13.8}</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:04.108407+00:00</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sp Gijon vs Burgos</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>23/08/2026 18:00</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>{"home": 42.9, "draw": 33.9, "away": 23.2}</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>{"home": 42.9, "draw": 33.9, "away": 23.2}</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:04.153573+00:00</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Tenerife vs Almeria</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>23/08/2026 20:30</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 17.7, "draw": 32.8, "away": 49.5}</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>{"home": 17.7, "draw": 32.8, "away": 49.5}</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-08-21T13:33:04.198259+00:00</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SP2</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Granada vs Mallorca</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>24/08/2026 20:30</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>1x2</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>{"home": 33.2, "draw": 35.3, "away": 31.5}</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>{"home": 33.2, "draw": 35.3, "away": 31.5}</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="A0A5"/>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>